<commit_message>
Milestone: Phase 5 - Compliance Dashboard & MongoDB Integration Complete
</commit_message>
<xml_diff>
--- a/docs/Man-Hours.xlsx
+++ b/docs/Man-Hours.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\agora-link\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB50883F-1CED-432A-9449-B349FAAA32AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42752BD6-58E9-4533-8ED8-8B96ADC6B119}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,10 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="30">
-  <si>
-    <t>Date</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="48">
   <si>
     <t>Task Description</t>
   </si>
@@ -39,9 +36,6 @@
     <t>Category</t>
   </si>
   <si>
-    <t>18-04-26</t>
-  </si>
-  <si>
     <t>Research: Garbled Circuits vs ZK-Proofs for Privacy</t>
   </si>
   <si>
@@ -66,9 +60,6 @@
     <t>Day 1 Total</t>
   </si>
   <si>
-    <t>19-04-26</t>
-  </si>
-  <si>
     <t>Feature Engineering &amp; Synthetic Data Generation</t>
   </si>
   <si>
@@ -93,12 +84,6 @@
     <t>Day 2 Total</t>
   </si>
   <si>
-    <t>Grand Total</t>
-  </si>
-  <si>
-    <t>20-04-26</t>
-  </si>
-  <si>
     <t>Node.js Gateway development &amp; ML Engine API integration</t>
   </si>
   <si>
@@ -115,13 +100,182 @@
   </si>
   <si>
     <t>Day 3 Total</t>
+  </si>
+  <si>
+    <r>
+      <t>Solidity smart contract drafting (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF444746"/>
+        <rFont val="Google Sans Text"/>
+        <family val="2"/>
+      </rPr>
+      <t>AgoraVault</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>) with access control</t>
+    </r>
+  </si>
+  <si>
+    <t>Testing edge cases for deposit/withdrawal on local Hardhat network</t>
+  </si>
+  <si>
+    <t>Deployment scripts creation and execution on Sepolia Testnet</t>
+  </si>
+  <si>
+    <t>Etherscan contract code verification and ABI extraction</t>
+  </si>
+  <si>
+    <t>Day 4 Total</t>
+  </si>
+  <si>
+    <r>
+      <t>ethers.js</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> integration in Node to interact with </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF444746"/>
+        <rFont val="Google Sans Text"/>
+        <family val="2"/>
+      </rPr>
+      <t>AgoraVault</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Private key management &amp; secure </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF444746"/>
+        <rFont val="Google Sans Text"/>
+        <family val="2"/>
+      </rPr>
+      <t>.env</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> configuration</t>
+    </r>
+  </si>
+  <si>
+    <t>Security</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Developing </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF444746"/>
+        <rFont val="Google Sans Text"/>
+        <family val="2"/>
+      </rPr>
+      <t>processBlockchainSettlement</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> payout function</t>
+    </r>
+  </si>
+  <si>
+    <t>Local E2E testing of Node.js calling Sepolia network</t>
+  </si>
+  <si>
+    <t>Day 5 Total</t>
+  </si>
+  <si>
+    <t>Vite + React repository initialization and dependency installation</t>
+  </si>
+  <si>
+    <t>Frontend</t>
+  </si>
+  <si>
+    <t>Custom CSS styling for dark-mode Fintech dashboard</t>
+  </si>
+  <si>
+    <t>Stripe Developer Account configuration and Test API Keys</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Stripe </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF444746"/>
+        <rFont val="Google Sans Text"/>
+        <family val="2"/>
+      </rPr>
+      <t>&lt;CardElement /&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF1F1F1F"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> integration for secure mock fiat input</t>
+    </r>
+  </si>
+  <si>
+    <t>Day 6 Total</t>
+  </si>
+  <si>
+    <t>CORS policy configuration and Express.js backend security updates</t>
+  </si>
+  <si>
+    <t>Dynamic fiat-to-USD mathematical conversion logic for Stripe</t>
+  </si>
+  <si>
+    <t>Axios POST requests bridging React UI with Node.js Gateway</t>
+  </si>
+  <si>
+    <t>Agentic UI state management (4-step status tracking &amp; receipt UI)</t>
+  </si>
+  <si>
+    <t>Day 7 Total</t>
+  </si>
+  <si>
+    <t>Total Sprint Hours</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -140,6 +294,12 @@
       <sz val="11"/>
       <color rgb="FF1F1F1F"/>
       <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF444746"/>
+      <name val="Google Sans Text"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -178,7 +338,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
@@ -191,6 +351,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -472,8 +635,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D17"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:D48"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="16.33203125" customWidth="1"/>
     <col min="2" max="2" width="28.33203125" customWidth="1"/>
@@ -481,233 +644,468 @@
     <col min="4" max="4" width="22.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:4" ht="15" thickBot="1">
+      <c r="A1" s="1"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+    </row>
+    <row r="2" spans="1:4" ht="21" customHeight="1" thickBot="1">
+      <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D2" s="4"/>
+    </row>
+    <row r="3" spans="1:4" ht="24.6" customHeight="1" thickBot="1">
+      <c r="A3" s="3" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="3" t="s">
+      <c r="B3" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="D3" s="4"/>
+    </row>
+    <row r="4" spans="1:4" ht="30" customHeight="1" thickBot="1">
+      <c r="A4" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="3">
-        <v>3.5</v>
-      </c>
-      <c r="D2" s="4" t="s">
+      <c r="B4" s="3">
+        <v>2.5</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4" s="4"/>
+    </row>
+    <row r="5" spans="1:4" ht="40.200000000000003" customHeight="1" thickBot="1">
+      <c r="A5" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" ht="24.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="3" t="s">
+      <c r="B5" s="3">
+        <v>2</v>
+      </c>
+      <c r="C5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="3">
+      <c r="D5" s="4"/>
+    </row>
+    <row r="6" spans="1:4" ht="69.599999999999994" thickBot="1">
+      <c r="A6" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="3">
+        <v>1</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" s="4"/>
+    </row>
+    <row r="7" spans="1:4" ht="15" thickBot="1">
+      <c r="A7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="1">
+        <v>9</v>
+      </c>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+    </row>
+    <row r="8" spans="1:4" ht="55.8" thickBot="1">
+      <c r="A8" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="3">
         <v>2.5</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" s="3">
-        <v>2</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="40.200000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" s="3">
-        <v>1</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" s="1" t="s">
+      <c r="C8" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="1">
-        <v>9</v>
-      </c>
-      <c r="D6" s="4"/>
-    </row>
-    <row r="7" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C7" s="3">
-        <v>2.5</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="42" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" s="3">
-        <v>3</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D8" s="4"/>
+    </row>
+    <row r="9" spans="1:4" ht="69.599999999999994" thickBot="1">
       <c r="A9" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="3">
+        <v>3</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" s="4"/>
+    </row>
+    <row r="10" spans="1:4" ht="55.8" thickBot="1">
+      <c r="A10" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="3">
+        <v>2</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D10" s="4"/>
+    </row>
+    <row r="11" spans="1:4" ht="69.599999999999994" thickBot="1">
+      <c r="A11" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11" s="3">
+        <v>1</v>
+      </c>
+      <c r="C11" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="3">
+      <c r="D11" s="4"/>
+    </row>
+    <row r="12" spans="1:4" ht="15" thickBot="1">
+      <c r="A12" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12" s="1">
+        <v>8.5</v>
+      </c>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+    </row>
+    <row r="13" spans="1:4" ht="69.599999999999994" thickBot="1">
+      <c r="A13" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B13" s="3">
+        <v>4</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D13" s="4"/>
+    </row>
+    <row r="14" spans="1:4" ht="55.8" thickBot="1">
+      <c r="A14" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" s="3">
+        <v>2.5</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D14" s="4"/>
+    </row>
+    <row r="15" spans="1:4" ht="69.599999999999994" thickBot="1">
+      <c r="A15" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B15" s="3">
+        <v>1</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D15" s="4"/>
+    </row>
+    <row r="16" spans="1:4" ht="69.599999999999994" thickBot="1">
+      <c r="A16" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B16" s="3">
+        <v>1</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D16" s="4"/>
+    </row>
+    <row r="17" spans="1:4" ht="15" thickBot="1">
+      <c r="A17" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B17" s="1">
+        <v>8.5</v>
+      </c>
+      <c r="C17" s="4"/>
+      <c r="D17" s="4"/>
+    </row>
+    <row r="18" spans="1:4" ht="83.4" thickBot="1">
+      <c r="A18" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B18" s="3">
+        <v>3</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="83.4" thickBot="1">
+      <c r="A19" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B19" s="3">
         <v>2</v>
       </c>
-      <c r="D9" s="4" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C10" s="3">
+      <c r="C19" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="69.599999999999994" thickBot="1">
+      <c r="A20" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B20" s="3">
+        <v>2.5</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="55.8" thickBot="1">
+      <c r="A21" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B21" s="3">
         <v>1</v>
       </c>
-      <c r="D10" s="4" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C11" s="1">
+      <c r="C21" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="15" thickBot="1">
+      <c r="A22" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B22" s="1">
         <v>8.5</v>
       </c>
-      <c r="D11" s="4"/>
-    </row>
-    <row r="12" spans="1:4" ht="42" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="C12" s="3">
-        <v>4</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="C13" s="3">
+      <c r="C22" s="4"/>
+    </row>
+    <row r="23" spans="1:4" ht="69" thickBot="1">
+      <c r="A23" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B23" s="3">
+        <v>3</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="55.8" thickBot="1">
+      <c r="A24" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B24" s="3">
+        <v>1.5</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="55.2" thickBot="1">
+      <c r="A25" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B25" s="3">
         <v>2.5</v>
       </c>
-      <c r="D13" s="4" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="42" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="C14" s="3">
+      <c r="C25" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="69.599999999999994" thickBot="1">
+      <c r="A26" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B26" s="3">
+        <v>1.5</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="15" thickBot="1">
+      <c r="A27" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B27" s="1">
+        <v>8.5</v>
+      </c>
+      <c r="C27" s="4"/>
+    </row>
+    <row r="28" spans="1:4" ht="83.4" thickBot="1">
+      <c r="A28" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B28" s="3">
         <v>1</v>
       </c>
-      <c r="D14" s="4" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="C15" s="3">
+      <c r="C28" s="4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="55.8" thickBot="1">
+      <c r="A29" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B29" s="3">
+        <v>2.5</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="83.4" thickBot="1">
+      <c r="A30" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B30" s="3">
         <v>1</v>
       </c>
-      <c r="D15" s="4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C16" s="1">
-        <v>8.5</v>
-      </c>
-      <c r="D16" s="4"/>
-    </row>
-    <row r="17" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B17" s="3"/>
-      <c r="C17" s="1">
-        <v>26</v>
-      </c>
-      <c r="D17" s="4"/>
+      <c r="C30" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" ht="69.599999999999994" thickBot="1">
+      <c r="A31" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B31" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="15" thickBot="1">
+      <c r="A32" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B32" s="1">
+        <v>8</v>
+      </c>
+      <c r="C32" s="4"/>
+    </row>
+    <row r="33" spans="1:3" ht="83.4" thickBot="1">
+      <c r="A33" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B33" s="3">
+        <v>1.5</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" ht="69.599999999999994" thickBot="1">
+      <c r="A34" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B34" s="3">
+        <v>2</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" ht="69.599999999999994" thickBot="1">
+      <c r="A35" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B35" s="3">
+        <v>2</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" ht="69.599999999999994" thickBot="1">
+      <c r="A36" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B36" s="3">
+        <v>2.5</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" ht="15" thickBot="1">
+      <c r="A37" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B37" s="1">
+        <v>8</v>
+      </c>
+      <c r="C37" s="4"/>
+    </row>
+    <row r="38" spans="1:3" ht="28.2" thickBot="1">
+      <c r="A38" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B38" s="1">
+        <v>59</v>
+      </c>
+      <c r="C38" s="4"/>
+    </row>
+    <row r="39" spans="1:3" ht="15" thickBot="1">
+      <c r="A39" s="3"/>
+      <c r="B39" s="3"/>
+      <c r="C39" s="4"/>
+    </row>
+    <row r="40" spans="1:3" ht="15" thickBot="1">
+      <c r="A40" s="3"/>
+      <c r="B40" s="3"/>
+      <c r="C40" s="4"/>
+    </row>
+    <row r="41" spans="1:3" ht="15" thickBot="1">
+      <c r="A41" s="3"/>
+      <c r="B41" s="3"/>
+      <c r="C41" s="4"/>
+    </row>
+    <row r="42" spans="1:3" ht="15" thickBot="1">
+      <c r="A42" s="1"/>
+      <c r="B42" s="1"/>
+      <c r="C42" s="4"/>
+    </row>
+    <row r="43" spans="1:3" ht="15" thickBot="1">
+      <c r="A43" s="3"/>
+      <c r="B43" s="3"/>
+      <c r="C43" s="4"/>
+    </row>
+    <row r="44" spans="1:3" ht="15" thickBot="1">
+      <c r="A44" s="3"/>
+      <c r="B44" s="3"/>
+      <c r="C44" s="4"/>
+    </row>
+    <row r="45" spans="1:3" ht="15" thickBot="1">
+      <c r="A45" s="3"/>
+      <c r="B45" s="3"/>
+      <c r="C45" s="4"/>
+    </row>
+    <row r="46" spans="1:3" ht="15" thickBot="1">
+      <c r="A46" s="3"/>
+      <c r="B46" s="3"/>
+      <c r="C46" s="4"/>
+    </row>
+    <row r="47" spans="1:3" ht="15" thickBot="1">
+      <c r="A47" s="1"/>
+      <c r="B47" s="1"/>
+      <c r="C47" s="4"/>
+    </row>
+    <row r="48" spans="1:3" ht="15" thickBot="1">
+      <c r="A48" s="1"/>
+      <c r="B48" s="1"/>
+      <c r="C48" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>